<commit_message>
post-processed pdf extractions. Manual highlights extracted for future reference.
</commit_message>
<xml_diff>
--- a/knowledge/models/system_of_interest_exploration.xlsx
+++ b/knowledge/models/system_of_interest_exploration.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\repos\capstone_isd\knowledge\models\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4002FAD5-40DB-458A-B08A-AE99B7194ECF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19E9983F-A9B9-41E5-8264-CF87E21F8E22}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="380" yWindow="0" windowWidth="21600" windowHeight="17370" xr2:uid="{EF918395-4981-400B-91E4-70C77FAFC499}"/>
   </bookViews>
@@ -822,7 +822,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:2" outlineLevel="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:2" hidden="1" outlineLevel="1" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>1</v>
       </c>
@@ -830,12 +830,12 @@
         <v>87</v>
       </c>
     </row>
-    <row r="4" spans="1:2" outlineLevel="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:2" hidden="1" outlineLevel="1" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="1:2" outlineLevel="2" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:2" hidden="1" outlineLevel="2" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
         <v>3</v>
       </c>
@@ -843,7 +843,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="6" spans="1:2" outlineLevel="2" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:2" hidden="1" outlineLevel="2" x14ac:dyDescent="0.35">
       <c r="A6" s="3" t="s">
         <v>4</v>
       </c>
@@ -852,7 +852,7 @@
         <v>information exchange between Dispatcher/ATC &amp; aircraft/crew</v>
       </c>
     </row>
-    <row r="7" spans="1:2" outlineLevel="2" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:2" hidden="1" outlineLevel="2" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
         <v>5</v>
       </c>
@@ -860,7 +860,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="8" spans="1:2" outlineLevel="2" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:2" hidden="1" outlineLevel="2" x14ac:dyDescent="0.35">
       <c r="A8" s="3" t="s">
         <v>6</v>
       </c>
@@ -868,7 +868,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="9" spans="1:2" outlineLevel="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:2" hidden="1" outlineLevel="1" collapsed="1" x14ac:dyDescent="0.35">
       <c r="A9" s="2" t="s">
         <v>91</v>
       </c>
@@ -876,7 +876,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="10" spans="1:2" outlineLevel="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:2" hidden="1" outlineLevel="1" x14ac:dyDescent="0.35">
       <c r="A10" s="2" t="s">
         <v>13</v>
       </c>
@@ -884,27 +884,27 @@
         <v>95</v>
       </c>
     </row>
-    <row r="11" spans="1:2" outlineLevel="2" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:2" hidden="1" outlineLevel="2" x14ac:dyDescent="0.35">
       <c r="A11" s="3" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="12" spans="1:2" outlineLevel="2" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:2" hidden="1" outlineLevel="2" x14ac:dyDescent="0.35">
       <c r="A12" s="3" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="13" spans="1:2" outlineLevel="2" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:2" hidden="1" outlineLevel="2" x14ac:dyDescent="0.35">
       <c r="A13" s="3" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="14" spans="1:2" outlineLevel="2" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:2" hidden="1" outlineLevel="2" x14ac:dyDescent="0.35">
       <c r="A14" s="3" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="15" spans="1:2" outlineLevel="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:2" hidden="1" outlineLevel="1" collapsed="1" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
         <v>17</v>
       </c>
@@ -912,7 +912,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="16" spans="1:2" outlineLevel="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:2" hidden="1" outlineLevel="1" x14ac:dyDescent="0.35">
       <c r="A16" s="2" t="s">
         <v>18</v>
       </c>
@@ -920,17 +920,17 @@
         <v>102</v>
       </c>
     </row>
-    <row r="17" spans="1:2" outlineLevel="2" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:2" hidden="1" outlineLevel="2" x14ac:dyDescent="0.35">
       <c r="A17" s="3" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="18" spans="1:2" outlineLevel="2" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:2" hidden="1" outlineLevel="2" x14ac:dyDescent="0.35">
       <c r="A18" s="3" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="19" spans="1:2" outlineLevel="2" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:2" hidden="1" outlineLevel="2" x14ac:dyDescent="0.35">
       <c r="A19" s="3" t="s">
         <v>21</v>
       </c>
@@ -938,7 +938,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="20" spans="1:2" outlineLevel="2" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:2" hidden="1" outlineLevel="2" x14ac:dyDescent="0.35">
       <c r="A20" s="3" t="s">
         <v>22</v>
       </c>
@@ -946,47 +946,47 @@
         <v>98</v>
       </c>
     </row>
-    <row r="21" spans="1:2" outlineLevel="2" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:2" hidden="1" outlineLevel="2" x14ac:dyDescent="0.35">
       <c r="A21" s="3" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="22" spans="1:2" outlineLevel="2" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:2" hidden="1" outlineLevel="2" x14ac:dyDescent="0.35">
       <c r="A22" s="3" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="23" spans="1:2" outlineLevel="2" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:2" hidden="1" outlineLevel="2" x14ac:dyDescent="0.35">
       <c r="A23" s="3" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="24" spans="1:2" outlineLevel="2" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:2" hidden="1" outlineLevel="2" x14ac:dyDescent="0.35">
       <c r="A24" s="3" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="25" spans="1:2" outlineLevel="2" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:2" hidden="1" outlineLevel="2" x14ac:dyDescent="0.35">
       <c r="A25" s="4" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="26" spans="1:2" outlineLevel="2" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:2" hidden="1" outlineLevel="2" x14ac:dyDescent="0.35">
       <c r="A26" s="4" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="27" spans="1:2" outlineLevel="2" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:2" hidden="1" outlineLevel="2" x14ac:dyDescent="0.35">
       <c r="A27" s="3" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="28" spans="1:2" outlineLevel="2" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:2" hidden="1" outlineLevel="2" x14ac:dyDescent="0.35">
       <c r="A28" s="3" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="29" spans="1:2" outlineLevel="2" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:2" hidden="1" outlineLevel="2" x14ac:dyDescent="0.35">
       <c r="A29" s="3" t="s">
         <v>31</v>
       </c>
@@ -994,7 +994,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="30" spans="1:2" outlineLevel="1" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:2" hidden="1" outlineLevel="1" collapsed="1" x14ac:dyDescent="0.35">
       <c r="A30" s="2" t="s">
         <v>32</v>
       </c>
@@ -1002,27 +1002,27 @@
         <v>104</v>
       </c>
     </row>
-    <row r="31" spans="1:2" outlineLevel="2" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:2" hidden="1" outlineLevel="2" x14ac:dyDescent="0.35">
       <c r="A31" s="3" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="32" spans="1:2" outlineLevel="2" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:2" hidden="1" outlineLevel="2" x14ac:dyDescent="0.35">
       <c r="A32" s="3" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="33" spans="1:2" outlineLevel="2" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:2" hidden="1" outlineLevel="2" x14ac:dyDescent="0.35">
       <c r="A33" s="3" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="34" spans="1:2" outlineLevel="2" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:2" hidden="1" outlineLevel="2" x14ac:dyDescent="0.35">
       <c r="A34" s="3" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="35" spans="1:2" outlineLevel="1" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:2" hidden="1" outlineLevel="1" collapsed="1" x14ac:dyDescent="0.35">
       <c r="A35" s="2" t="s">
         <v>37</v>
       </c>
@@ -1030,22 +1030,22 @@
         <v>106</v>
       </c>
     </row>
-    <row r="36" spans="1:2" outlineLevel="2" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:2" hidden="1" outlineLevel="2" x14ac:dyDescent="0.35">
       <c r="A36" s="3" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="37" spans="1:2" outlineLevel="2" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:2" hidden="1" outlineLevel="2" x14ac:dyDescent="0.35">
       <c r="A37" s="3" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="38" spans="1:2" outlineLevel="2" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:2" hidden="1" outlineLevel="2" x14ac:dyDescent="0.35">
       <c r="A38" s="3" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="39" spans="1:2" outlineLevel="1" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:2" hidden="1" outlineLevel="1" collapsed="1" x14ac:dyDescent="0.35">
       <c r="A39" s="2" t="s">
         <v>40</v>
       </c>
@@ -1053,7 +1053,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="40" spans="1:2" outlineLevel="1" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:2" hidden="1" outlineLevel="1" x14ac:dyDescent="0.35">
       <c r="A40" s="2" t="s">
         <v>41</v>
       </c>
@@ -1061,7 +1061,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="41" spans="1:2" outlineLevel="1" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:2" hidden="1" outlineLevel="1" x14ac:dyDescent="0.35">
       <c r="A41" s="2" t="s">
         <v>42</v>
       </c>
@@ -1069,22 +1069,22 @@
         <v>108</v>
       </c>
     </row>
-    <row r="42" spans="1:2" outlineLevel="2" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:2" hidden="1" outlineLevel="2" x14ac:dyDescent="0.35">
       <c r="A42" s="3" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="43" spans="1:2" outlineLevel="2" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:2" hidden="1" outlineLevel="2" x14ac:dyDescent="0.35">
       <c r="A43" s="3" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="44" spans="1:2" outlineLevel="2" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:2" hidden="1" outlineLevel="2" x14ac:dyDescent="0.35">
       <c r="A44" s="3" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:2" collapsed="1" x14ac:dyDescent="0.35">
       <c r="A45" s="5" t="s">
         <v>7</v>
       </c>
@@ -1092,7 +1092,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="46" spans="1:2" outlineLevel="1" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:2" hidden="1" outlineLevel="1" x14ac:dyDescent="0.35">
       <c r="A46" s="1" t="s">
         <v>8</v>
       </c>
@@ -1101,7 +1101,7 @@
         <v>Takes actions to control aircraft to achieve objective.</v>
       </c>
     </row>
-    <row r="47" spans="1:2" outlineLevel="1" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:2" hidden="1" outlineLevel="1" x14ac:dyDescent="0.35">
       <c r="A47" s="1" t="s">
         <v>9</v>
       </c>
@@ -1110,7 +1110,7 @@
         <v>Takes actions to control aircraft to achieve objective.</v>
       </c>
     </row>
-    <row r="48" spans="1:2" outlineLevel="1" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:2" hidden="1" outlineLevel="1" x14ac:dyDescent="0.35">
       <c r="A48" s="1" t="s">
         <v>10</v>
       </c>
@@ -1119,7 +1119,7 @@
         <v>Takes actions to control aircraft to achieve objective.</v>
       </c>
     </row>
-    <row r="49" spans="1:2" outlineLevel="1" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:2" hidden="1" outlineLevel="1" x14ac:dyDescent="0.35">
       <c r="A49" s="1" t="s">
         <v>11</v>
       </c>
@@ -1128,7 +1128,7 @@
         <v>Takes actions to control aircraft to achieve objective.</v>
       </c>
     </row>
-    <row r="50" spans="1:2" outlineLevel="1" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:2" hidden="1" outlineLevel="1" x14ac:dyDescent="0.35">
       <c r="A50" s="1" t="s">
         <v>12</v>
       </c>
@@ -1136,7 +1136,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="51" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:2" collapsed="1" x14ac:dyDescent="0.35">
       <c r="A51" s="5" t="s">
         <v>46</v>
       </c>
@@ -1152,22 +1152,22 @@
         <v>110</v>
       </c>
     </row>
-    <row r="53" spans="1:2" outlineLevel="1" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:2" hidden="1" outlineLevel="1" x14ac:dyDescent="0.35">
       <c r="A53" s="2" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="54" spans="1:2" outlineLevel="1" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:2" hidden="1" outlineLevel="1" x14ac:dyDescent="0.35">
       <c r="A54" s="2" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="55" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:2" collapsed="1" x14ac:dyDescent="0.35">
       <c r="A55" s="5" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="56" spans="1:2" outlineLevel="1" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:2" hidden="1" outlineLevel="1" x14ac:dyDescent="0.35">
       <c r="A56" s="2" t="s">
         <v>50</v>
       </c>
@@ -1175,7 +1175,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="57" spans="1:2" outlineLevel="1" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:2" hidden="1" outlineLevel="1" x14ac:dyDescent="0.35">
       <c r="A57" s="2" t="s">
         <v>112</v>
       </c>
@@ -1183,27 +1183,27 @@
         <v>113</v>
       </c>
     </row>
-    <row r="58" spans="1:2" outlineLevel="2" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:2" hidden="1" outlineLevel="2" x14ac:dyDescent="0.35">
       <c r="A58" s="3" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="59" spans="1:2" outlineLevel="2" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:2" hidden="1" outlineLevel="2" x14ac:dyDescent="0.35">
       <c r="A59" s="3" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="60" spans="1:2" outlineLevel="2" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:2" hidden="1" outlineLevel="2" x14ac:dyDescent="0.35">
       <c r="A60" s="3" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="61" spans="1:2" outlineLevel="2" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:2" hidden="1" outlineLevel="2" x14ac:dyDescent="0.35">
       <c r="A61" s="3" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="62" spans="1:2" outlineLevel="1" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:2" hidden="1" outlineLevel="1" collapsed="1" x14ac:dyDescent="0.35">
       <c r="A62" s="2" t="s">
         <v>55</v>
       </c>
@@ -1211,7 +1211,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="63" spans="1:2" outlineLevel="1" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:2" hidden="1" outlineLevel="1" x14ac:dyDescent="0.35">
       <c r="A63" s="2" t="s">
         <v>56</v>
       </c>
@@ -1219,7 +1219,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="64" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:2" collapsed="1" x14ac:dyDescent="0.35">
       <c r="A64" s="5" t="s">
         <v>57</v>
       </c>
@@ -1227,7 +1227,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="65" spans="1:2" outlineLevel="1" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:2" hidden="1" outlineLevel="1" x14ac:dyDescent="0.35">
       <c r="A65" s="2" t="s">
         <v>58</v>
       </c>
@@ -1235,7 +1235,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="66" spans="1:2" outlineLevel="1" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:2" hidden="1" outlineLevel="1" x14ac:dyDescent="0.35">
       <c r="A66" s="2" t="s">
         <v>59</v>
       </c>
@@ -1243,7 +1243,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="67" spans="1:2" outlineLevel="1" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:2" hidden="1" outlineLevel="1" x14ac:dyDescent="0.35">
       <c r="A67" s="2" t="s">
         <v>60</v>
       </c>
@@ -1251,7 +1251,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="68" spans="1:2" outlineLevel="1" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:2" hidden="1" outlineLevel="1" x14ac:dyDescent="0.35">
       <c r="A68" s="2" t="s">
         <v>61</v>
       </c>
@@ -1259,7 +1259,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="69" spans="1:2" outlineLevel="1" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:2" hidden="1" outlineLevel="1" x14ac:dyDescent="0.35">
       <c r="A69" s="2" t="s">
         <v>62</v>
       </c>
@@ -1267,12 +1267,12 @@
         <v>119</v>
       </c>
     </row>
-    <row r="70" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:2" collapsed="1" x14ac:dyDescent="0.35">
       <c r="A70" s="5" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="71" spans="1:2" outlineLevel="1" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:2" hidden="1" outlineLevel="1" x14ac:dyDescent="0.35">
       <c r="A71" s="2" t="s">
         <v>64</v>
       </c>
@@ -1280,7 +1280,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="72" spans="1:2" outlineLevel="1" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:2" hidden="1" outlineLevel="1" x14ac:dyDescent="0.35">
       <c r="A72" s="2" t="s">
         <v>65</v>
       </c>
@@ -1288,7 +1288,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="73" spans="1:2" outlineLevel="2" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:2" hidden="1" outlineLevel="2" x14ac:dyDescent="0.35">
       <c r="A73" s="3" t="s">
         <v>66</v>
       </c>
@@ -1296,7 +1296,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="74" spans="1:2" outlineLevel="2" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:2" hidden="1" outlineLevel="2" x14ac:dyDescent="0.35">
       <c r="A74" s="3" t="s">
         <v>67</v>
       </c>
@@ -1304,7 +1304,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="75" spans="1:2" outlineLevel="2" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:2" hidden="1" outlineLevel="2" x14ac:dyDescent="0.35">
       <c r="A75" s="3" t="s">
         <v>8</v>
       </c>
@@ -1312,7 +1312,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="76" spans="1:2" outlineLevel="2" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:2" hidden="1" outlineLevel="2" x14ac:dyDescent="0.35">
       <c r="A76" s="3" t="s">
         <v>68</v>
       </c>
@@ -1320,7 +1320,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="77" spans="1:2" outlineLevel="2" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:2" hidden="1" outlineLevel="2" x14ac:dyDescent="0.35">
       <c r="A77" s="3" t="s">
         <v>69</v>
       </c>
@@ -1328,7 +1328,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="78" spans="1:2" outlineLevel="2" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:2" hidden="1" outlineLevel="2" x14ac:dyDescent="0.35">
       <c r="A78" s="3" t="s">
         <v>70</v>
       </c>
@@ -1336,7 +1336,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="79" spans="1:2" outlineLevel="1" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:2" hidden="1" outlineLevel="1" collapsed="1" x14ac:dyDescent="0.35">
       <c r="A79" s="2" t="s">
         <v>71</v>
       </c>
@@ -1344,7 +1344,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="80" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:2" collapsed="1" x14ac:dyDescent="0.35">
       <c r="A80" s="5" t="s">
         <v>72</v>
       </c>
@@ -1352,7 +1352,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="81" spans="1:2" outlineLevel="1" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:2" hidden="1" outlineLevel="1" x14ac:dyDescent="0.35">
       <c r="A81" s="2" t="s">
         <v>73</v>
       </c>
@@ -1360,7 +1360,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="82" spans="1:2" outlineLevel="2" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:2" hidden="1" outlineLevel="2" x14ac:dyDescent="0.35">
       <c r="A82" s="3" t="s">
         <v>74</v>
       </c>
@@ -1368,7 +1368,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="83" spans="1:2" outlineLevel="2" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:2" hidden="1" outlineLevel="2" x14ac:dyDescent="0.35">
       <c r="A83" s="3" t="s">
         <v>75</v>
       </c>
@@ -1376,17 +1376,17 @@
         <v>127</v>
       </c>
     </row>
-    <row r="84" spans="1:2" outlineLevel="1" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:2" hidden="1" outlineLevel="1" collapsed="1" x14ac:dyDescent="0.35">
       <c r="A84" s="2" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="85" spans="1:2" outlineLevel="2" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:2" hidden="1" outlineLevel="2" x14ac:dyDescent="0.35">
       <c r="A85" s="3" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="86" spans="1:2" outlineLevel="2" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:2" hidden="1" outlineLevel="2" x14ac:dyDescent="0.35">
       <c r="A86" s="3" t="s">
         <v>78</v>
       </c>
@@ -1394,12 +1394,12 @@
         <v>128</v>
       </c>
     </row>
-    <row r="87" spans="1:2" outlineLevel="2" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:2" hidden="1" outlineLevel="2" x14ac:dyDescent="0.35">
       <c r="A87" s="3" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="88" spans="1:2" outlineLevel="2" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:2" hidden="1" outlineLevel="2" x14ac:dyDescent="0.35">
       <c r="A88" s="3" t="s">
         <v>80</v>
       </c>
@@ -1407,7 +1407,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="89" spans="1:2" outlineLevel="2" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:2" hidden="1" outlineLevel="2" x14ac:dyDescent="0.35">
       <c r="A89" s="3" t="s">
         <v>81</v>
       </c>
@@ -1415,7 +1415,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="90" spans="1:2" outlineLevel="2" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:2" hidden="1" outlineLevel="2" x14ac:dyDescent="0.35">
       <c r="A90" s="3" t="s">
         <v>82</v>
       </c>
@@ -1423,7 +1423,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="91" spans="1:2" outlineLevel="2" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:2" hidden="1" outlineLevel="2" x14ac:dyDescent="0.35">
       <c r="A91" s="3" t="s">
         <v>83</v>
       </c>
@@ -1431,7 +1431,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="92" spans="1:2" outlineLevel="1" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:2" hidden="1" outlineLevel="1" collapsed="1" x14ac:dyDescent="0.35">
       <c r="A92" s="2" t="s">
         <v>84</v>
       </c>
@@ -1439,7 +1439,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="93" spans="1:2" outlineLevel="1" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:2" hidden="1" outlineLevel="1" x14ac:dyDescent="0.35">
       <c r="A93" s="2" t="s">
         <v>85</v>
       </c>
@@ -1447,7 +1447,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="94" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:2" collapsed="1" x14ac:dyDescent="0.35">
       <c r="A94" s="5" t="s">
         <v>86</v>
       </c>

</xml_diff>